<commit_message>
Configuraciones finales sobre caso de REMOFIRST que tiene 2 secciones en el excel, se configuran los correos de yuly y viviana para el envio de correos
</commit_message>
<xml_diff>
--- a/Facturación REMOFIRST - Septiembre.xlsx
+++ b/Facturación REMOFIRST - Septiembre.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F860EFE-7E26-4BE6-A6E2-8B65309EDF54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1C3F4DA-4A0F-4417-A41F-AD0B3A71CE70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1864" uniqueCount="692">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1863" uniqueCount="691">
   <si>
     <t>Etiquetas de fila</t>
   </si>
@@ -2113,9 +2113,6 @@
   </si>
   <si>
     <t>2820</t>
-  </si>
-  <si>
-    <t>VALOR TOTAL FACTURA EN USD</t>
   </si>
 </sst>
 </file>
@@ -37771,33 +37768,16 @@
       </c>
     </row>
     <row r="180" spans="1:70" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="BH180" s="64">
-        <f>+SUM(M4:AE168,AI4:AN168,AR4:AT168,AX4:BC168,M172:AE177,AI172:AN177,AR172:AT177,AX172:BC177)</f>
-        <v>1706932840</v>
-      </c>
-      <c r="BN180" s="65">
-        <f>+SUM(BN169,BN178)</f>
-        <v>566897.80000000016</v>
-      </c>
-      <c r="BQ180" s="62">
-        <f>BQ169+BQ178</f>
-        <v>578678.80000000005</v>
-      </c>
-      <c r="BR180" s="63" t="s">
-        <v>691</v>
-      </c>
+      <c r="BH180" s="64"/>
+      <c r="BN180" s="65"/>
+      <c r="BQ180" s="62"/>
+      <c r="BR180" s="63"/>
     </row>
     <row r="182" spans="1:70" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="BH182" s="64">
-        <f>+SUM(BH180,BI169:BK169,BJ178)</f>
-        <v>1749375123.4099998</v>
-      </c>
+      <c r="BH182" s="64"/>
     </row>
     <row r="184" spans="1:70" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="BH184" s="65">
-        <f>+BH182/BM177</f>
-        <v>578678.85857329506</v>
-      </c>
+      <c r="BH184" s="65"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>